<commit_message>
Swap the Digital LED buck to the ME3116
The LGS5145 refused to start below 5.2 V on the bench, a full volt above
the 4.2 V UVLO its datasheet gives, so a 5 V PSU never brought the rail up.
Its frequency fold-back at low feedback voltage is the likely reason: at
start-up FB is low by definition, and with little input headroom the part
never gathers enough volt-seconds to leave the hiccup.

The ME3116 is a drop-in - same SOT23-6 pinout, and with a 0.8 V reference
instead of 0.812 V the existing 51k/10k divider lands at 4.88 V. Measured
4.44 V out at 5 V in, which clears the 3.5 V the strip needs on its data
line, so one assembly now covers 5 V to 24 V and R7 stays not fitted.
</commit_message>
<xml_diff>
--- a/Hardware/DALI_Load_250W_DigitalLED/JLC_PCBA_CPL-DALI_LOAD_DigitalLED(V0.1).xlsx
+++ b/Hardware/DALI_Load_250W_DigitalLED/JLC_PCBA_CPL-DALI_LOAD_DigitalLED(V0.1).xlsx
@@ -228,7 +228,7 @@
     <t>10.795</t>
   </si>
   <si>
-    <t>1.25A</t>
+    <t>0.8A</t>
   </si>
   <si>
     <t>1808 Fuse / FUSE_0154004</t>
@@ -255,7 +255,7 @@
     <t>12</t>
   </si>
   <si>
-    <t>LGS5145</t>
+    <t>ME3116</t>
   </si>
   <si>
     <t>SOT95P280X110-6N (SOT23-6L)</t>

</xml_diff>

<commit_message>
Digital LED board: 250 V rated mains fuse
F1 was a Littelfuse 0154 in 1808, rated 125 V only. Replaced by a 1032
ceramic SMD fuse rated 250 V. The old part sat in a holder, so the
footprint stays practically the same. Fab outputs regenerated, ODB++ added.
</commit_message>
<xml_diff>
--- a/Hardware/DALI_Load_250W_DigitalLED/JLC_PCBA_CPL-DALI_LOAD_DigitalLED(V0.1).xlsx
+++ b/Hardware/DALI_Load_250W_DigitalLED/JLC_PCBA_CPL-DALI_LOAD_DigitalLED(V0.1).xlsx
@@ -222,16 +222,16 @@
     <t>F1</t>
   </si>
   <si>
-    <t>19.736</t>
-  </si>
-  <si>
-    <t>10.795</t>
+    <t>19.749</t>
+  </si>
+  <si>
+    <t>11.036</t>
   </si>
   <si>
     <t>0.8A</t>
   </si>
   <si>
-    <t>1808 Fuse / FUSE_0154004</t>
+    <t>FUSE-SMD_L10.3-W3.2</t>
   </si>
   <si>
     <t>FB1</t>

</xml_diff>